<commit_message>
Use development version of camtrapdp Correct inspection modifs Remove the sound of norway link
</commit_message>
<xml_diff>
--- a/datasets/maryland/data/interim/table_comparison.xlsx
+++ b/datasets/maryland/data/interim/table_comparison.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="211">
   <si>
     <t xml:space="preserve">arrayName</t>
   </si>
@@ -237,106 +237,103 @@
     <t xml:space="preserve">Spectrogram </t>
   </si>
   <si>
-    <t xml:space="preserve">3878915.699971</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3878921.516021</t>
+    <t xml:space="preserve">1847375.851978</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1847381.668028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">08/01/2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180801\86896MD01_016K_M04_multi_20180801_211500Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180801_211500Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">575.851978105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21:24:35.852</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.509177</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1-4-f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">parm file = FW2O_p25.mat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018-08-01T21:15:00+00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180801_211500Z_14463</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Balaenoptera physalus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">95567.315971</t>
+  </si>
+  <si>
+    <t xml:space="preserve">95573.132021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07/12/2018</t>
+  </si>
+  <si>
+    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180712\86896MD01_016K_M04_multi_20180712_144500Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180712_144500Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">167.315971399</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14:47:47.316</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.619703</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018-07-12T14:45:00+00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180712_144500Z_3608</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3883273.883978</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3883279.700028</t>
   </si>
   <si>
     <t xml:space="preserve">08/25/2018</t>
   </si>
   <si>
-    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180825\86896MD01_016K_M04_multi_20180825_093000Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180825_093000Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">815.699971399</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09:43:35.700</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.550667</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1-4-f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">parm file = FW2O_p25.mat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2018-08-25T09:30:00+00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180825_093000Z_38425</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Balaenoptera physalus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3576950.963145</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3576955.020855</t>
-  </si>
-  <si>
-    <t xml:space="preserve">08/21/2018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180821\86896MD01_016K_M04_multi_20180821_214500Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180821_214500Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">350.963145176</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21:50:50.963</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.564352</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1-2-f</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2018-08-21T21:45:00+00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180821_214500Z_30396</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1309582.843978</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1309588.660028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07/26/2018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180726\86896MD01_016K_M04_multi_20180726_160000Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180726_160000Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">82.843978105</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16:01:22.844</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.561526</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2018-07-26T16:00:00+00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180726_160000Z_11819</t>
+    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180825\86896MD01_016K_M04_multi_20180825_104500Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180825_104500Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">673.883978105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:56:13.884</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.577402</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018-08-25T10:45:00+00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180825_104500Z_38525</t>
   </si>
   <si>
     <t xml:space="preserve">locationID</t>
@@ -486,37 +483,37 @@
     <t xml:space="preserve">mediaComments</t>
   </si>
   <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180818_154500Z.aif</t>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180818_160000Z.aif</t>
   </si>
   <si>
     <t xml:space="preserve">schedule</t>
   </si>
   <si>
-    <t xml:space="preserve">2018-08-18T15:45:00+00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180818\86896MD01_016K_M04_multi_20180818_154500Z.aif</t>
+    <t xml:space="preserve">2018-08-18T16:00:00+00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180818\86896MD01_016K_M04_multi_20180818_160000Z.aif</t>
   </si>
   <si>
     <t xml:space="preserve">audio/aiff</t>
   </si>
   <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180819_163000Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2018-08-19T16:30:00+00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180819\86896MD01_016K_M04_multi_20180819_163000Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180712_003000Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2018-07-12T00:30:00+00:00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180712\86896MD01_016K_M04_multi_20180712_003000Z.aif</t>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180819_103000Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018-08-19T10:30:00+00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180819\86896MD01_016K_M04_multi_20180819_103000Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180712_111500Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018-07-12T11:15:00+00:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">\\Repnas\w\projects\2018_UnivMD_Maryland_86896\86896_MD01_20180711\86896_MD01_AIFF\86896MD01_016K_M04_multi_20180712\86896MD01_016K_M04_multi_20180712_111500Z.aif</t>
   </si>
   <si>
     <t xml:space="preserve">eventID</t>
@@ -600,16 +597,16 @@
     <t xml:space="preserve">observationComments</t>
   </si>
   <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180821_224500Z_30492</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180821_224500Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3580406.595149</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3580410.652859</t>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180822_210000Z_31730</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180822_210000Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3660999.483975</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3661005.300025</t>
   </si>
   <si>
     <t xml:space="preserve">interval</t>
@@ -621,37 +618,37 @@
     <t xml:space="preserve">machine</t>
   </si>
   <si>
-    <t xml:space="preserve">0.662134</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180725_193000Z_11418</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180725_193000Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1236085.659975</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1236091.476025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.530456</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180715_163000Z_5776</t>
-  </si>
-  <si>
-    <t xml:space="preserve">86896MD01_016K_M04_multi_20180715_163000Z.aif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">361406.739975</t>
-  </si>
-  <si>
-    <t xml:space="preserve">361412.556025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.508256</t>
+    <t xml:space="preserve">0.528144</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180728_151500Z_12761</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180728_151500Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1479864.075978</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1479869.892028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.526975</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180720_041500Z_7989</t>
+  </si>
+  <si>
+    <t xml:space="preserve">86896MD01_016K_M04_multi_20180720_041500Z.aif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">749249.651971</t>
+  </si>
+  <si>
+    <t xml:space="preserve">749255.468021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.548584</t>
   </si>
 </sst>
 </file>
@@ -1543,16 +1540,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>38425</v>
+        <v>14463</v>
       </c>
       <c r="B2" t="s">
         <v>72</v>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" t="s">
         <v>73</v>
@@ -1570,7 +1567,7 @@
         <v>75</v>
       </c>
       <c r="J2" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="K2" t="s">
         <v>76</v>
@@ -1611,16 +1608,16 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>30396</v>
+        <v>3608</v>
       </c>
       <c r="B3" t="s">
         <v>72</v>
       </c>
       <c r="C3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" t="s">
         <v>86</v>
@@ -1632,13 +1629,13 @@
         <v>13</v>
       </c>
       <c r="H3" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="I3" t="s">
         <v>88</v>
       </c>
       <c r="J3" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="K3" t="s">
         <v>89</v>
@@ -1659,7 +1656,7 @@
         <v>93</v>
       </c>
       <c r="Q3" t="s">
-        <v>94</v>
+        <v>81</v>
       </c>
       <c r="R3" t="s">
         <v>82</v>
@@ -1668,10 +1665,10 @@
         <v>45</v>
       </c>
       <c r="T3" t="s">
+        <v>94</v>
+      </c>
+      <c r="U3" t="s">
         <v>95</v>
-      </c>
-      <c r="U3" t="s">
-        <v>96</v>
       </c>
       <c r="V3" t="s">
         <v>85</v>
@@ -1679,7 +1676,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>11819</v>
+        <v>38525</v>
       </c>
       <c r="B4" t="s">
         <v>72</v>
@@ -1691,10 +1688,10 @@
         <v>3</v>
       </c>
       <c r="E4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" t="s">
         <v>97</v>
-      </c>
-      <c r="F4" t="s">
-        <v>98</v>
       </c>
       <c r="G4" t="n">
         <v>13</v>
@@ -1703,28 +1700,28 @@
         <v>29</v>
       </c>
       <c r="I4" t="s">
+        <v>98</v>
+      </c>
+      <c r="J4" t="n">
+        <v>10</v>
+      </c>
+      <c r="K4" t="s">
         <v>99</v>
       </c>
-      <c r="J4" t="n">
-        <v>16</v>
-      </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>100</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>101</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
+        <v>98</v>
+      </c>
+      <c r="O4" t="s">
         <v>102</v>
       </c>
-      <c r="N4" t="s">
-        <v>99</v>
-      </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>103</v>
-      </c>
-      <c r="P4" t="s">
-        <v>104</v>
       </c>
       <c r="Q4" t="s">
         <v>81</v>
@@ -1736,10 +1733,10 @@
         <v>45</v>
       </c>
       <c r="T4" t="s">
+        <v>104</v>
+      </c>
+      <c r="U4" t="s">
         <v>105</v>
-      </c>
-      <c r="U4" t="s">
-        <v>106</v>
       </c>
       <c r="V4" t="s">
         <v>85</v>
@@ -1761,79 +1758,79 @@
         <v>68</v>
       </c>
       <c r="B1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1" t="s">
         <v>107</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>108</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>109</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>110</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>111</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>112</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>113</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>114</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>115</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>116</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>117</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>118</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>119</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>120</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>121</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>122</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>123</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>124</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>125</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>126</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>127</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>128</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>129</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>130</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="2">
@@ -1841,7 +1838,7 @@
         <v>45</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C2"/>
       <c r="D2" t="n">
@@ -1853,10 +1850,10 @@
       <c r="F2"/>
       <c r="G2"/>
       <c r="H2" t="s">
+        <v>132</v>
+      </c>
+      <c r="I2" t="s">
         <v>133</v>
-      </c>
-      <c r="I2" t="s">
-        <v>134</v>
       </c>
       <c r="J2"/>
       <c r="K2" t="n">
@@ -1866,7 +1863,7 @@
         <v>40</v>
       </c>
       <c r="M2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N2"/>
       <c r="O2"/>
@@ -1876,7 +1873,7 @@
       <c r="Q2"/>
       <c r="R2"/>
       <c r="S2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="T2"/>
       <c r="U2"/>
@@ -1887,7 +1884,7 @@
       </c>
       <c r="Y2"/>
       <c r="Z2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3">
@@ -1907,10 +1904,10 @@
       <c r="F3"/>
       <c r="G3"/>
       <c r="H3" t="s">
+        <v>137</v>
+      </c>
+      <c r="I3" t="s">
         <v>138</v>
-      </c>
-      <c r="I3" t="s">
-        <v>139</v>
       </c>
       <c r="J3"/>
       <c r="K3" t="n">
@@ -1920,7 +1917,7 @@
         <v>40</v>
       </c>
       <c r="M3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N3"/>
       <c r="O3"/>
@@ -1930,7 +1927,7 @@
       <c r="Q3"/>
       <c r="R3"/>
       <c r="S3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="T3"/>
       <c r="U3"/>
@@ -1961,10 +1958,10 @@
       <c r="F4"/>
       <c r="G4"/>
       <c r="H4" t="s">
+        <v>139</v>
+      </c>
+      <c r="I4" t="s">
         <v>140</v>
-      </c>
-      <c r="I4" t="s">
-        <v>141</v>
       </c>
       <c r="J4"/>
       <c r="K4" t="n">
@@ -1974,7 +1971,7 @@
         <v>40</v>
       </c>
       <c r="M4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="N4"/>
       <c r="O4"/>
@@ -1984,7 +1981,7 @@
       <c r="Q4"/>
       <c r="R4"/>
       <c r="S4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="T4"/>
       <c r="U4"/>
@@ -2009,77 +2006,77 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B1" t="s">
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D1" t="s">
         <v>69</v>
       </c>
       <c r="E1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F1" t="s">
         <v>144</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>145</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>146</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>147</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>148</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>149</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>150</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>151</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>152</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>153</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>154</v>
-      </c>
-      <c r="P1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B2" t="s">
         <v>45</v>
       </c>
       <c r="C2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D2" t="s">
         <v>157</v>
-      </c>
-      <c r="D2" t="s">
-        <v>158</v>
       </c>
       <c r="E2"/>
       <c r="F2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G2" t="b">
         <v>0</v>
       </c>
       <c r="H2"/>
       <c r="I2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J2"/>
       <c r="K2" t="n">
@@ -2097,27 +2094,27 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B3" t="s">
         <v>45</v>
       </c>
       <c r="C3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E3"/>
       <c r="F3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G3" t="b">
         <v>0</v>
       </c>
       <c r="H3"/>
       <c r="I3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J3"/>
       <c r="K3" t="n">
@@ -2135,27 +2132,27 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B4" t="s">
         <v>45</v>
       </c>
       <c r="C4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E4"/>
       <c r="F4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G4" t="b">
         <v>0</v>
       </c>
       <c r="H4"/>
       <c r="I4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J4"/>
       <c r="K4" t="n">
@@ -2190,115 +2187,115 @@
         <v>68</v>
       </c>
       <c r="C1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E1" t="s">
         <v>167</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>168</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>169</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>170</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>171</v>
-      </c>
-      <c r="I1" t="s">
-        <v>172</v>
       </c>
       <c r="J1" t="s">
         <v>71</v>
       </c>
       <c r="K1" t="s">
+        <v>172</v>
+      </c>
+      <c r="L1" t="s">
         <v>173</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>174</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>175</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>176</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>177</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>178</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>179</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>180</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>181</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>182</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>183</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>184</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>185</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>186</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>187</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>188</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>189</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>190</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AD1" t="s">
         <v>191</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AE1" t="s">
         <v>192</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" t="s">
         <v>45</v>
       </c>
       <c r="C2" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D2"/>
       <c r="E2" t="s">
+        <v>195</v>
+      </c>
+      <c r="F2" t="s">
         <v>196</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>197</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>198</v>
-      </c>
-      <c r="H2" t="s">
-        <v>199</v>
       </c>
       <c r="I2"/>
       <c r="J2" t="s">
@@ -2319,12 +2316,12 @@
       <c r="W2"/>
       <c r="X2"/>
       <c r="Y2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="Z2"/>
       <c r="AA2"/>
       <c r="AB2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="AC2"/>
       <c r="AD2"/>
@@ -2334,26 +2331,26 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B3" t="s">
         <v>45</v>
       </c>
       <c r="C3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D3"/>
       <c r="E3" t="s">
+        <v>203</v>
+      </c>
+      <c r="F3" t="s">
         <v>204</v>
       </c>
-      <c r="F3" t="s">
-        <v>205</v>
-      </c>
       <c r="G3" t="s">
+        <v>197</v>
+      </c>
+      <c r="H3" t="s">
         <v>198</v>
-      </c>
-      <c r="H3" t="s">
-        <v>199</v>
       </c>
       <c r="I3"/>
       <c r="J3" t="s">
@@ -2374,12 +2371,12 @@
       <c r="W3"/>
       <c r="X3"/>
       <c r="Y3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="Z3"/>
       <c r="AA3"/>
       <c r="AB3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AC3"/>
       <c r="AD3"/>
@@ -2389,26 +2386,26 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B4" t="s">
         <v>45</v>
       </c>
       <c r="C4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D4"/>
       <c r="E4" t="s">
+        <v>208</v>
+      </c>
+      <c r="F4" t="s">
         <v>209</v>
       </c>
-      <c r="F4" t="s">
-        <v>210</v>
-      </c>
       <c r="G4" t="s">
+        <v>197</v>
+      </c>
+      <c r="H4" t="s">
         <v>198</v>
-      </c>
-      <c r="H4" t="s">
-        <v>199</v>
       </c>
       <c r="I4"/>
       <c r="J4" t="s">
@@ -2429,12 +2426,12 @@
       <c r="W4"/>
       <c r="X4"/>
       <c r="Y4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="Z4"/>
       <c r="AA4"/>
       <c r="AB4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="AC4"/>
       <c r="AD4"/>

</xml_diff>